<commit_message>
Stabilization of Belgium Rehire - In Progress
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Belgium_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Belgium_Regression_PK14.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{ED5B066C-472B-4B39-9A99-13125A6718E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DC2AF1-639C-493A-94A0-D878EA778AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +11,6 @@
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="209">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -232,7 +231,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10698379</t>
+    <t>10698458</t>
   </si>
   <si>
     <t>Passed</t>
@@ -250,7 +249,7 @@
     <t>BelgiumOne</t>
   </si>
   <si>
-    <t>TwentyFiveJuneTwoA</t>
+    <t>TwentyFiveJuneNineA</t>
   </si>
   <si>
     <t>Landline</t>
@@ -382,7 +381,7 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10698380</t>
+    <t>Failed</t>
   </si>
   <si>
     <t>751 Store Management (Mupol Bypitu (10528834))</t>
@@ -394,10 +393,10 @@
     <t>BelgiumTwo</t>
   </si>
   <si>
-    <t>TwentyFiveJuneTwo</t>
-  </si>
-  <si>
-    <t>Auto 87634024</t>
+    <t>TwentyFiveJuneNine</t>
+  </si>
+  <si>
+    <t>Auto 66285002</t>
   </si>
   <si>
     <t>Fixed Term</t>
@@ -424,9 +423,6 @@
     <t>Test3</t>
   </si>
   <si>
-    <t>10698381</t>
-  </si>
-  <si>
     <t>BelgiumThree</t>
   </si>
   <si>
@@ -445,13 +441,10 @@
     <t>Test4</t>
   </si>
   <si>
-    <t>10698382</t>
-  </si>
-  <si>
     <t>BelgiumFour</t>
   </si>
   <si>
-    <t>Auto 59586408</t>
+    <t>Auto 28143044</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -466,7 +459,7 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>10698383</t>
+    <t>10698462</t>
   </si>
   <si>
     <t>BelgiumFive</t>
@@ -484,13 +477,10 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>10698384</t>
-  </si>
-  <si>
     <t>BelgiumSix</t>
   </si>
   <si>
-    <t>Auto 92877324</t>
+    <t>Auto 21896146</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -505,13 +495,10 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>10698385</t>
-  </si>
-  <si>
     <t>BelgiumSeven</t>
   </si>
   <si>
-    <t>Auto 47827197</t>
+    <t>Auto 49758543</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -526,13 +513,10 @@
     <t>Test8</t>
   </si>
   <si>
-    <t>10698386</t>
-  </si>
-  <si>
     <t>BelgiumEight</t>
   </si>
   <si>
-    <t>Auto 68051437</t>
+    <t>Auto 48512271</t>
   </si>
   <si>
     <t>Visual Merchandising Manager_NEW</t>
@@ -547,7 +531,7 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10698387</t>
+    <t>10698466</t>
   </si>
   <si>
     <t>BelgiumNineReRun</t>
@@ -571,7 +555,7 @@
     <t>Test10</t>
   </si>
   <si>
-    <t>10698388</t>
+    <t>10698467</t>
   </si>
   <si>
     <t>BelgiumTen</t>
@@ -592,7 +576,7 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10698390</t>
+    <t>10698468</t>
   </si>
   <si>
     <t>BelgiumEleven</t>
@@ -610,7 +594,7 @@
     <t>Test12</t>
   </si>
   <si>
-    <t>10698391</t>
+    <t>10698469</t>
   </si>
   <si>
     <t>BelgiumTweleve</t>
@@ -631,7 +615,7 @@
     <t>Test13</t>
   </si>
   <si>
-    <t>10698393</t>
+    <t>10698470</t>
   </si>
   <si>
     <t>BelgiumThirteen</t>
@@ -649,15 +633,12 @@
     <t>Test14</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'BelgiumFourteen TwentyFiveJuneTwo' Employee:{Mupol Bypitu }TimeoutError: locator.click: Timeout 30000ms exceeded.
+    <t xml:space="preserve">Test failed for 'BelgiumFourteen TwentyFiveJuneNine' Employee:{Mupol Bypitu }TimeoutError: locator.click: Timeout 30000ms exceeded.
 Call log:
-  [2m- waiting for locator('text=Onboarding Guide: In-Store P&amp;C Assistant_NEW - BelgiumFourteen TwentyFiveJuneTwo')[22m
+  [2m- waiting for locator('text=Onboarding Guide: In-Store P&amp;C Assistant_NEW - BelgiumFourteen TwentyFiveJuneNine')[22m
 </t>
   </si>
   <si>
-    <t>Failed</t>
-  </si>
-  <si>
     <t>BelgiumFourteen</t>
   </si>
   <si>
@@ -670,13 +651,10 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>10698394</t>
-  </si>
-  <si>
     <t>BelgiumFifteen</t>
   </si>
   <si>
-    <t>Auto 93363956</t>
+    <t>Auto 26294116</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -753,7 +731,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
@@ -1611,7 +1589,7 @@
       </c>
       <c r="L2" s="19">
         <f t="shared" ref="L2:L16" ca="1" si="0">TODAY()-31</f>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M2" s="14" t="s">
         <v>70</v>
@@ -1645,7 +1623,7 @@
       </c>
       <c r="W2" s="22">
         <f t="shared" ref="W2:W16" ca="1" si="1">L2</f>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X2" s="18" t="s">
         <v>81</v>
@@ -1697,7 +1675,7 @@
       </c>
       <c r="AN2" s="1">
         <f t="array" aca="1" ref="AN2" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>69715006575</v>
+        <v>68862601559</v>
       </c>
       <c r="AO2" s="14" t="s">
         <v>94</v>
@@ -1792,8 +1770,8 @@
       <c r="A3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>117</v>
+      <c r="B3" s="11">
+        <v>10698459</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>68</v>
@@ -1824,7 +1802,7 @@
       </c>
       <c r="L3" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M3" s="14" t="s">
         <v>70</v>
@@ -1858,7 +1836,7 @@
       </c>
       <c r="W3" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X3" s="18" t="s">
         <v>81</v>
@@ -1892,7 +1870,7 @@
       </c>
       <c r="AH3" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AI3" s="18" t="s">
         <v>90</v>
@@ -1911,7 +1889,7 @@
       </c>
       <c r="AN3" s="1">
         <f t="array" aca="1" ref="AN3" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>92965956429</v>
+        <v>93994314052</v>
       </c>
       <c r="AO3" s="14" t="s">
         <v>94</v>
@@ -1924,7 +1902,7 @@
       </c>
       <c r="AR3" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AS3" s="24" t="s">
         <v>127</v>
@@ -2006,8 +1984,8 @@
       <c r="A4" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>131</v>
+      <c r="B4" s="11">
+        <v>10698460</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>68</v>
@@ -2022,7 +2000,7 @@
         <v>71</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>121</v>
@@ -2038,7 +2016,7 @@
       </c>
       <c r="L4" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M4" s="14" t="s">
         <v>70</v>
@@ -2072,7 +2050,7 @@
       </c>
       <c r="W4" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X4" s="18" t="s">
         <v>81</v>
@@ -2084,10 +2062,10 @@
         <v>83</v>
       </c>
       <c r="AA4" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="AB4" s="24" t="s">
         <v>133</v>
-      </c>
-      <c r="AB4" s="24" t="s">
-        <v>134</v>
       </c>
       <c r="AC4" s="24" t="s">
         <v>86</v>
@@ -2114,7 +2092,7 @@
         <v>91</v>
       </c>
       <c r="AK4" s="24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AL4" s="27" t="s">
         <v>70</v>
@@ -2124,7 +2102,7 @@
       </c>
       <c r="AN4" s="1">
         <f t="array" aca="1" ref="AN4" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>28127547886</v>
+        <v>21779498096</v>
       </c>
       <c r="AO4" s="14" t="s">
         <v>94</v>
@@ -2209,7 +2187,7 @@
         <v>114</v>
       </c>
       <c r="BP4" s="32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="BQ4" s="33">
         <v>100</v>
@@ -2217,10 +2195,10 @@
     </row>
     <row r="5" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>138</v>
+        <v>136</v>
+      </c>
+      <c r="B5" s="11">
+        <v>10698461</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>68</v>
@@ -2235,7 +2213,7 @@
         <v>119</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>121</v>
@@ -2251,7 +2229,7 @@
       </c>
       <c r="L5" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M5" s="14" t="s">
         <v>70</v>
@@ -2285,19 +2263,19 @@
       </c>
       <c r="W5" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X5" s="18" t="s">
         <v>81</v>
       </c>
       <c r="Y5" s="23" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="Z5" s="24" t="s">
         <v>83</v>
       </c>
       <c r="AA5" s="25" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AB5" s="24" t="s">
         <v>85</v>
@@ -2337,7 +2315,7 @@
       </c>
       <c r="AN5" s="1">
         <f t="array" aca="1" ref="AN5" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>90300131870</v>
+        <v>36457753212</v>
       </c>
       <c r="AO5" s="14" t="s">
         <v>94</v>
@@ -2380,10 +2358,10 @@
         <v>70</v>
       </c>
       <c r="BB5" s="34" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="BC5" s="24" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="BD5" s="14" t="s">
         <v>103</v>
@@ -2430,10 +2408,10 @@
     </row>
     <row r="6" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>68</v>
@@ -2448,7 +2426,7 @@
         <v>71</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>121</v>
@@ -2464,7 +2442,7 @@
       </c>
       <c r="L6" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M6" s="14" t="s">
         <v>70</v>
@@ -2498,7 +2476,7 @@
       </c>
       <c r="W6" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X6" s="18" t="s">
         <v>81</v>
@@ -2507,13 +2485,13 @@
         <v>82</v>
       </c>
       <c r="Z6" s="24" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AA6" s="25" t="s">
         <v>84</v>
       </c>
       <c r="AB6" s="24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC6" s="24" t="s">
         <v>86</v>
@@ -2532,7 +2510,7 @@
       </c>
       <c r="AH6" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AI6" s="18" t="s">
         <v>90</v>
@@ -2541,7 +2519,7 @@
         <v>91</v>
       </c>
       <c r="AK6" s="24" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="AL6" s="27" t="s">
         <v>70</v>
@@ -2551,7 +2529,7 @@
       </c>
       <c r="AN6" s="1">
         <f t="array" aca="1" ref="AN6" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>58479723927</v>
+        <v>43444326011</v>
       </c>
       <c r="AO6" s="14" t="s">
         <v>94</v>
@@ -2564,7 +2542,7 @@
       </c>
       <c r="AR6" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AS6" s="24" t="s">
         <v>97</v>
@@ -2636,7 +2614,7 @@
         <v>114</v>
       </c>
       <c r="BP6" s="32" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="BQ6" s="33">
         <v>100</v>
@@ -2644,10 +2622,10 @@
     </row>
     <row r="7" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>151</v>
+        <v>148</v>
+      </c>
+      <c r="B7" s="11">
+        <v>10698463</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>68</v>
@@ -2662,7 +2640,7 @@
         <v>71</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>121</v>
@@ -2678,7 +2656,7 @@
       </c>
       <c r="L7" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M7" s="14" t="s">
         <v>70</v>
@@ -2712,22 +2690,22 @@
       </c>
       <c r="W7" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X7" s="18" t="s">
         <v>81</v>
       </c>
       <c r="Y7" s="23" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Z7" s="36" t="s">
         <v>83</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="AB7" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC7" s="24" t="s">
         <v>86</v>
@@ -2764,7 +2742,7 @@
       </c>
       <c r="AN7" s="1">
         <f t="array" aca="1" ref="AN7" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>77611762933</v>
+        <v>29197137746</v>
       </c>
       <c r="AO7" s="14" t="s">
         <v>94</v>
@@ -2807,10 +2785,10 @@
         <v>70</v>
       </c>
       <c r="BB7" s="24" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="BC7" s="24" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="BD7" s="14" t="s">
         <v>103</v>
@@ -2849,7 +2827,7 @@
         <v>114</v>
       </c>
       <c r="BP7" s="32" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="BQ7" s="33">
         <v>100</v>
@@ -2857,10 +2835,10 @@
     </row>
     <row r="8" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
+      </c>
+      <c r="B8" s="11">
+        <v>10698464</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>68</v>
@@ -2875,7 +2853,7 @@
         <v>71</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>121</v>
@@ -2891,7 +2869,7 @@
       </c>
       <c r="L8" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M8" s="14" t="s">
         <v>70</v>
@@ -2925,19 +2903,19 @@
       </c>
       <c r="W8" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X8" s="18" t="s">
         <v>81</v>
       </c>
       <c r="Y8" s="23" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="Z8" s="36" t="s">
         <v>123</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="AB8" s="37" t="s">
         <v>85</v>
@@ -2959,7 +2937,7 @@
       </c>
       <c r="AH8" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AI8" s="18" t="s">
         <v>90</v>
@@ -2978,7 +2956,7 @@
       </c>
       <c r="AN8" s="1">
         <f t="array" aca="1" ref="AN8" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>94591458563</v>
+        <v>28141011648</v>
       </c>
       <c r="AO8" s="14" t="s">
         <v>94</v>
@@ -2991,7 +2969,7 @@
       </c>
       <c r="AR8" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AS8" s="24" t="s">
         <v>97</v>
@@ -3021,10 +2999,10 @@
         <v>70</v>
       </c>
       <c r="BB8" s="24" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="BC8" s="24" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="BD8" s="14" t="s">
         <v>103</v>
@@ -3071,10 +3049,10 @@
     </row>
     <row r="9" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>165</v>
+        <v>160</v>
+      </c>
+      <c r="B9" s="11">
+        <v>10698465</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>68</v>
@@ -3089,7 +3067,7 @@
         <v>71</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>121</v>
@@ -3105,7 +3083,7 @@
       </c>
       <c r="L9" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M9" s="14" t="s">
         <v>70</v>
@@ -3139,22 +3117,22 @@
       </c>
       <c r="W9" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X9" s="18" t="s">
         <v>81</v>
       </c>
       <c r="Y9" s="23" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="Z9" s="36" t="s">
         <v>83</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="AB9" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC9" s="24" t="s">
         <v>86</v>
@@ -3191,7 +3169,7 @@
       </c>
       <c r="AN9" s="1">
         <f t="array" aca="1" ref="AN9" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>45146593568</v>
+        <v>88781270421</v>
       </c>
       <c r="AO9" s="14" t="s">
         <v>94</v>
@@ -3234,10 +3212,10 @@
         <v>70</v>
       </c>
       <c r="BB9" s="24" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="BC9" s="24" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="BD9" s="14" t="s">
         <v>103</v>
@@ -3276,7 +3254,7 @@
         <v>114</v>
       </c>
       <c r="BP9" s="32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="BQ9" s="33">
         <v>100</v>
@@ -3284,10 +3262,10 @@
     </row>
     <row r="10" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>68</v>
@@ -3302,7 +3280,7 @@
         <v>71</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>121</v>
@@ -3318,7 +3296,7 @@
       </c>
       <c r="L10" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M10" s="14" t="s">
         <v>70</v>
@@ -3352,7 +3330,7 @@
       </c>
       <c r="W10" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X10" s="18" t="s">
         <v>81</v>
@@ -3361,19 +3339,19 @@
         <v>82</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="AB10" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC10" s="24" t="s">
         <v>86</v>
       </c>
       <c r="AD10" s="24" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
@@ -3386,7 +3364,7 @@
       </c>
       <c r="AH10" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AI10" s="18" t="s">
         <v>90</v>
@@ -3395,7 +3373,7 @@
         <v>91</v>
       </c>
       <c r="AK10" s="24" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="AL10" s="27" t="s">
         <v>70</v>
@@ -3405,20 +3383,20 @@
       </c>
       <c r="AN10" s="1">
         <f t="array" aca="1" ref="AN10" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>64184169355</v>
+        <v>97580190593</v>
       </c>
       <c r="AO10" s="14" t="s">
         <v>94</v>
       </c>
       <c r="AP10" s="18" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="AQ10" s="18" t="s">
         <v>96</v>
       </c>
       <c r="AR10" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AS10" s="24" t="s">
         <v>97</v>
@@ -3490,7 +3468,7 @@
         <v>114</v>
       </c>
       <c r="BP10" s="32" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="BQ10" s="33">
         <v>100</v>
@@ -3498,10 +3476,10 @@
     </row>
     <row r="11" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>68</v>
@@ -3516,7 +3494,7 @@
         <v>71</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>121</v>
@@ -3532,7 +3510,7 @@
       </c>
       <c r="L11" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M11" s="14" t="s">
         <v>70</v>
@@ -3566,7 +3544,7 @@
       </c>
       <c r="W11" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X11" s="18" t="s">
         <v>81</v>
@@ -3578,7 +3556,7 @@
         <v>83</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="AB11" s="34" t="s">
         <v>85</v>
@@ -3608,7 +3586,7 @@
         <v>91</v>
       </c>
       <c r="AK11" s="24" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="AL11" s="27" t="s">
         <v>70</v>
@@ -3618,7 +3596,7 @@
       </c>
       <c r="AN11" s="1">
         <f t="array" aca="1" ref="AN11" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>57216194164</v>
+        <v>44661214921</v>
       </c>
       <c r="AO11" s="14" t="s">
         <v>94</v>
@@ -3661,10 +3639,10 @@
         <v>70</v>
       </c>
       <c r="BB11" s="24" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="BC11" s="24" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="BD11" s="14" t="s">
         <v>103</v>
@@ -3711,10 +3689,10 @@
     </row>
     <row r="12" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>68</v>
@@ -3729,7 +3707,7 @@
         <v>71</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>121</v>
@@ -3745,7 +3723,7 @@
       </c>
       <c r="L12" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M12" s="14" t="s">
         <v>70</v>
@@ -3779,7 +3757,7 @@
       </c>
       <c r="W12" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X12" s="18" t="s">
         <v>81</v>
@@ -3791,10 +3769,10 @@
         <v>83</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="AB12" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC12" s="24" t="s">
         <v>86</v>
@@ -3821,7 +3799,7 @@
         <v>91</v>
       </c>
       <c r="AK12" s="24" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="AL12" s="27" t="s">
         <v>70</v>
@@ -3831,7 +3809,7 @@
       </c>
       <c r="AN12" s="1">
         <f t="array" aca="1" ref="AN12" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>85087577396</v>
+        <v>47336777057</v>
       </c>
       <c r="AO12" s="14" t="s">
         <v>94</v>
@@ -3916,7 +3894,7 @@
         <v>114</v>
       </c>
       <c r="BP12" s="32" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="BQ12" s="33">
         <v>100</v>
@@ -3924,10 +3902,10 @@
     </row>
     <row r="13" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>68</v>
@@ -3942,7 +3920,7 @@
         <v>71</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>121</v>
@@ -3958,7 +3936,7 @@
       </c>
       <c r="L13" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M13" s="14" t="s">
         <v>70</v>
@@ -3992,7 +3970,7 @@
       </c>
       <c r="W13" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X13" s="18" t="s">
         <v>81</v>
@@ -4004,7 +3982,7 @@
         <v>123</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="AB13" s="37" t="s">
         <v>85</v>
@@ -4026,7 +4004,7 @@
       </c>
       <c r="AH13" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AI13" s="18" t="s">
         <v>90</v>
@@ -4035,7 +4013,7 @@
         <v>91</v>
       </c>
       <c r="AK13" s="24" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="AL13" s="27" t="s">
         <v>70</v>
@@ -4045,7 +4023,7 @@
       </c>
       <c r="AN13" s="1">
         <f t="array" aca="1" ref="AN13" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>40161645789</v>
+        <v>28957789980</v>
       </c>
       <c r="AO13" s="14" t="s">
         <v>94</v>
@@ -4058,7 +4036,7 @@
       </c>
       <c r="AR13" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AS13" s="24" t="s">
         <v>97</v>
@@ -4088,10 +4066,10 @@
         <v>70</v>
       </c>
       <c r="BB13" s="24" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="BD13" s="14" t="s">
         <v>103</v>
@@ -4138,10 +4116,10 @@
     </row>
     <row r="14" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>68</v>
@@ -4156,7 +4134,7 @@
         <v>71</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>121</v>
@@ -4172,7 +4150,7 @@
       </c>
       <c r="L14" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M14" s="14" t="s">
         <v>70</v>
@@ -4206,7 +4184,7 @@
       </c>
       <c r="W14" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X14" s="18" t="s">
         <v>81</v>
@@ -4218,10 +4196,10 @@
         <v>83</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="AB14" s="37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AC14" s="24" t="s">
         <v>86</v>
@@ -4248,7 +4226,7 @@
         <v>91</v>
       </c>
       <c r="AK14" s="34" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="AL14" s="27" t="s">
         <v>70</v>
@@ -4258,7 +4236,7 @@
       </c>
       <c r="AN14" s="1">
         <f t="array" aca="1" ref="AN14" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>66824185657</v>
+        <v>51349978822</v>
       </c>
       <c r="AO14" s="14" t="s">
         <v>94</v>
@@ -4343,7 +4321,7 @@
         <v>114</v>
       </c>
       <c r="BP14" s="32" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="BQ14" s="33">
         <v>100</v>
@@ -4351,13 +4329,13 @@
     </row>
     <row r="15" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>207</v>
+        <v>117</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>69</v>
@@ -4369,7 +4347,7 @@
         <v>71</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="H15" s="17" t="s">
         <v>121</v>
@@ -4385,7 +4363,7 @@
       </c>
       <c r="L15" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M15" s="14" t="s">
         <v>70</v>
@@ -4419,7 +4397,7 @@
       </c>
       <c r="W15" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X15" s="18" t="s">
         <v>81</v>
@@ -4431,10 +4409,10 @@
         <v>123</v>
       </c>
       <c r="AA15" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="AB15" s="37" t="s">
         <v>133</v>
-      </c>
-      <c r="AB15" s="37" t="s">
-        <v>134</v>
       </c>
       <c r="AC15" s="24" t="s">
         <v>86</v>
@@ -4453,7 +4431,7 @@
       </c>
       <c r="AH15" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AI15" s="18" t="s">
         <v>90</v>
@@ -4462,7 +4440,7 @@
         <v>91</v>
       </c>
       <c r="AK15" s="24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AL15" s="27" t="s">
         <v>70</v>
@@ -4472,7 +4450,7 @@
       </c>
       <c r="AN15" s="1">
         <f t="array" aca="1" ref="AN15" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>99059206105</v>
+        <v>98582859372</v>
       </c>
       <c r="AO15" s="14" t="s">
         <v>94</v>
@@ -4485,7 +4463,7 @@
       </c>
       <c r="AR15" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46175</v>
+        <v>46183</v>
       </c>
       <c r="AS15" s="24" t="s">
         <v>97</v>
@@ -4515,10 +4493,10 @@
         <v>70</v>
       </c>
       <c r="BB15" s="24" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="BC15" s="24" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="BD15" s="14" t="s">
         <v>103</v>
@@ -4557,7 +4535,7 @@
         <v>114</v>
       </c>
       <c r="BP15" s="32" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="BQ15" s="33">
         <v>100</v>
@@ -4565,10 +4543,10 @@
     </row>
     <row r="16" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>212</v>
+        <v>205</v>
+      </c>
+      <c r="B16" s="11">
+        <v>10698471</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>68</v>
@@ -4583,7 +4561,7 @@
         <v>71</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>121</v>
@@ -4599,7 +4577,7 @@
       </c>
       <c r="L16" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="M16" s="14" t="s">
         <v>70</v>
@@ -4633,19 +4611,19 @@
       </c>
       <c r="W16" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45779</v>
+        <v>45787</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>81</v>
       </c>
       <c r="Y16" s="23" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="Z16" s="34" t="s">
         <v>83</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="AB16" s="37" t="s">
         <v>85</v>
@@ -4685,7 +4663,7 @@
       </c>
       <c r="AN16" s="1">
         <f t="array" aca="1" ref="AN16" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>16331790509</v>
+        <v>53875782183</v>
       </c>
       <c r="AO16" s="14" t="s">
         <v>94</v>
@@ -4803,7 +4781,7 @@
     <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId16"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Poland and Belgium Rehire completed 24th June
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Belgium_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Belgium_Regression_PK14.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DC2AF1-639C-493A-94A0-D878EA778AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{8E87A658-16E8-4432-87C5-BC9D13EE7B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,6 +11,7 @@
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="220">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -228,10 +229,13 @@
     <t>AllowanceAmount</t>
   </si>
   <si>
+    <t>EducationLevel</t>
+  </si>
+  <si>
     <t>Test1</t>
   </si>
   <si>
-    <t>10698458</t>
+    <t>10698599</t>
   </si>
   <si>
     <t>Passed</t>
@@ -249,7 +253,7 @@
     <t>BelgiumOne</t>
   </si>
   <si>
-    <t>TwentyFiveJuneNineA</t>
+    <t>TwentyFiveJuneTwentyThreeA</t>
   </si>
   <si>
     <t>Landline</t>
@@ -294,7 +298,7 @@
     <t>V2 BIS - (Job Qualifications-Belgium)</t>
   </si>
   <si>
-    <t>5 Days (Belgium)</t>
+    <t>5 Days</t>
   </si>
   <si>
     <t>N/A</t>
@@ -378,267 +382,294 @@
     <t>Variable | 35 | A35</t>
   </si>
   <si>
+    <t>Primary School</t>
+  </si>
+  <si>
     <t>Test2</t>
   </si>
   <si>
+    <t>10698612</t>
+  </si>
+  <si>
+    <t>751 Store Management (Mupol Bypitu (10528834))</t>
+  </si>
+  <si>
+    <t>Mme</t>
+  </si>
+  <si>
+    <t>BelgiumTwo</t>
+  </si>
+  <si>
+    <t>Auto 79650253</t>
+  </si>
+  <si>
+    <t>Fixed Term</t>
+  </si>
+  <si>
+    <t>Store Manager_NEW</t>
+  </si>
+  <si>
+    <t>V2 - (Job Qualifications-Belgium)</t>
+  </si>
+  <si>
+    <t>92 Retail</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Belgium Retail - Store Manager (1st Store, 2nd Store, 3rd store)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store Manager - First Store </t>
+  </si>
+  <si>
+    <t>Secondary School</t>
+  </si>
+  <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>10698601</t>
+  </si>
+  <si>
+    <t>BelgiumThree</t>
+  </si>
+  <si>
+    <t>TwentyFiveJuneTwentyThree</t>
+  </si>
+  <si>
+    <t>In-Store P&amp;C Assistant_NEW</t>
+  </si>
+  <si>
+    <t>Part time</t>
+  </si>
+  <si>
+    <t>250 Human Resources Retail</t>
+  </si>
+  <si>
+    <t>Variable | 20 | A20</t>
+  </si>
+  <si>
+    <t>Non-university Higher Education</t>
+  </si>
+  <si>
+    <t>Test4</t>
+  </si>
+  <si>
+    <t>10698602</t>
+  </si>
+  <si>
+    <t>BelgiumFour</t>
+  </si>
+  <si>
+    <t>Auto 3183499</t>
+  </si>
+  <si>
+    <t>Team Manager - Retail_NEW</t>
+  </si>
+  <si>
+    <t>Belgium Retail - Team Manager</t>
+  </si>
+  <si>
+    <t>Team Manager</t>
+  </si>
+  <si>
+    <t>University</t>
+  </si>
+  <si>
+    <t>Test5</t>
+  </si>
+  <si>
+    <t>10698603</t>
+  </si>
+  <si>
+    <t>BelgiumFive</t>
+  </si>
+  <si>
+    <t>06 Menswear</t>
+  </si>
+  <si>
+    <t>Variable | 30 | A30</t>
+  </si>
+  <si>
+    <t>Test6</t>
+  </si>
+  <si>
+    <t>10698604</t>
+  </si>
+  <si>
+    <t>BelgiumSix</t>
+  </si>
+  <si>
+    <t>Auto 83744345</t>
+  </si>
+  <si>
+    <t>Department Manager_NEW</t>
+  </si>
+  <si>
+    <t>Belgium Retail - Dpt. Manager</t>
+  </si>
+  <si>
+    <t>Department Manager</t>
+  </si>
+  <si>
+    <t>Test7</t>
+  </si>
+  <si>
+    <t>10698613</t>
+  </si>
+  <si>
+    <t>BelgiumSeven</t>
+  </si>
+  <si>
+    <t>Auto 7357027</t>
+  </si>
+  <si>
+    <t>Assistant Store Manager_NEW</t>
+  </si>
+  <si>
+    <t>Belgium Retail - Assistant Manager</t>
+  </si>
+  <si>
+    <t>Assistant Manager</t>
+  </si>
+  <si>
+    <t>Test8</t>
+  </si>
+  <si>
+    <t>10698605</t>
+  </si>
+  <si>
+    <t>BelgiumEight</t>
+  </si>
+  <si>
+    <t>Auto 78378810</t>
+  </si>
+  <si>
+    <t>Visual Merchandising Manager_NEW</t>
+  </si>
+  <si>
+    <t>Belgium Retail - VM (entry / junior (after 3 months) / experienced)</t>
+  </si>
+  <si>
+    <t>VM (Entry)</t>
+  </si>
+  <si>
+    <t>Test9</t>
+  </si>
+  <si>
+    <t>10698606</t>
+  </si>
+  <si>
+    <t>BelgiumNine</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Retail Assistant Special Contracts_NEW</t>
+  </si>
+  <si>
+    <t>Hourly</t>
+  </si>
+  <si>
+    <t>260 Fitting Rooms</t>
+  </si>
+  <si>
+    <t>Variable | 10 | A10</t>
+  </si>
+  <si>
+    <t>Test10</t>
+  </si>
+  <si>
+    <t>10698607</t>
+  </si>
+  <si>
+    <t>BelgiumTen</t>
+  </si>
+  <si>
+    <t>Retail Assistant Cash Office_NEW</t>
+  </si>
+  <si>
+    <t>258 Cash Office</t>
+  </si>
+  <si>
+    <t>Belgium Category III - Experience 10</t>
+  </si>
+  <si>
+    <t>CAT III 3 Year Seniority</t>
+  </si>
+  <si>
+    <t>Test11</t>
+  </si>
+  <si>
+    <t>10698608</t>
+  </si>
+  <si>
+    <t>BelgiumEleven</t>
+  </si>
+  <si>
+    <t>Supervisor_NEW</t>
+  </si>
+  <si>
+    <t>253 Supervisors</t>
+  </si>
+  <si>
+    <t>Variable | 28 | A28</t>
+  </si>
+  <si>
+    <t>Test12</t>
+  </si>
+  <si>
+    <t>10698609</t>
+  </si>
+  <si>
+    <t>BelgiumTweleve</t>
+  </si>
+  <si>
+    <t>Visual Merchandiser_NEW</t>
+  </si>
+  <si>
+    <t>256 Visual Merchandising</t>
+  </si>
+  <si>
+    <t>Belgium Retail - Visual Merchandiser - Experience 1</t>
+  </si>
+  <si>
+    <t>CAT III 1 Year Seniority</t>
+  </si>
+  <si>
+    <t>Test13</t>
+  </si>
+  <si>
+    <t>10698610</t>
+  </si>
+  <si>
+    <t>BelgiumThirteen</t>
+  </si>
+  <si>
+    <t>Supervisor Stockroom_NEW</t>
+  </si>
+  <si>
+    <t>255 Stockroom</t>
+  </si>
+  <si>
+    <t>Variable | 20 | A20/4</t>
+  </si>
+  <si>
+    <t>Test14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test failed for 'BelgiumFourteen TwentyFiveJuneTwentyThree' Employee:{Mupol Bypitu }TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for locator('//div[@data-automation-id=\'titleText\'][contains(./text(),\'Hire: BelgiumFourteen TwentyFiveJuneTwentyThree\')]').first()[22m
+</t>
+  </si>
+  <si>
     <t>Failed</t>
   </si>
   <si>
-    <t>751 Store Management (Mupol Bypitu (10528834))</t>
-  </si>
-  <si>
-    <t>Mme</t>
-  </si>
-  <si>
-    <t>BelgiumTwo</t>
-  </si>
-  <si>
-    <t>TwentyFiveJuneNine</t>
-  </si>
-  <si>
-    <t>Auto 66285002</t>
-  </si>
-  <si>
-    <t>Fixed Term</t>
-  </si>
-  <si>
-    <t>Store Manager_NEW</t>
-  </si>
-  <si>
-    <t>V2 - (Job Qualifications-Belgium)</t>
-  </si>
-  <si>
-    <t>92 Retail</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Belgium Retail - Store Manager (1st Store, 2nd Store, 3rd store)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store Manager - First Store </t>
-  </si>
-  <si>
-    <t>Test3</t>
-  </si>
-  <si>
-    <t>BelgiumThree</t>
-  </si>
-  <si>
-    <t>In-Store P&amp;C Assistant_NEW</t>
-  </si>
-  <si>
-    <t>Part time</t>
-  </si>
-  <si>
-    <t>250 Human Resources Retail</t>
-  </si>
-  <si>
-    <t>Variable | 20 | A20</t>
-  </si>
-  <si>
-    <t>Test4</t>
-  </si>
-  <si>
-    <t>BelgiumFour</t>
-  </si>
-  <si>
-    <t>Auto 28143044</t>
-  </si>
-  <si>
-    <t>Team Manager - Retail_NEW</t>
-  </si>
-  <si>
-    <t>Belgium Retail - Team Manager</t>
-  </si>
-  <si>
-    <t>Team Manager</t>
-  </si>
-  <si>
-    <t>Test5</t>
-  </si>
-  <si>
-    <t>10698462</t>
-  </si>
-  <si>
-    <t>BelgiumFive</t>
-  </si>
-  <si>
-    <t>Intern</t>
-  </si>
-  <si>
-    <t>06 Menswear</t>
-  </si>
-  <si>
-    <t>Variable | 30 | A30</t>
-  </si>
-  <si>
-    <t>Test6</t>
-  </si>
-  <si>
-    <t>BelgiumSix</t>
-  </si>
-  <si>
-    <t>Auto 21896146</t>
-  </si>
-  <si>
-    <t>Department Manager_NEW</t>
-  </si>
-  <si>
-    <t>Belgium Retail - Dpt. Manager</t>
-  </si>
-  <si>
-    <t>Department Manager</t>
-  </si>
-  <si>
-    <t>Test7</t>
-  </si>
-  <si>
-    <t>BelgiumSeven</t>
-  </si>
-  <si>
-    <t>Auto 49758543</t>
-  </si>
-  <si>
-    <t>Assistant Store Manager_NEW</t>
-  </si>
-  <si>
-    <t>Belgium Retail - Assistant Manager</t>
-  </si>
-  <si>
-    <t>Assistant Manager</t>
-  </si>
-  <si>
-    <t>Test8</t>
-  </si>
-  <si>
-    <t>BelgiumEight</t>
-  </si>
-  <si>
-    <t>Auto 48512271</t>
-  </si>
-  <si>
-    <t>Visual Merchandising Manager_NEW</t>
-  </si>
-  <si>
-    <t>Belgium Retail - VM (entry / junior (after 3 months) / experienced)</t>
-  </si>
-  <si>
-    <t>VM (Entry)</t>
-  </si>
-  <si>
-    <t>Test9</t>
-  </si>
-  <si>
-    <t>10698466</t>
-  </si>
-  <si>
-    <t>BelgiumNineReRun</t>
-  </si>
-  <si>
-    <t>Students</t>
-  </si>
-  <si>
-    <t>Retail Assistant Special Contracts_NEW</t>
-  </si>
-  <si>
-    <t>Hourly</t>
-  </si>
-  <si>
-    <t>260 Fitting Rooms</t>
-  </si>
-  <si>
-    <t>Variable | 10 | A10</t>
-  </si>
-  <si>
-    <t>Test10</t>
-  </si>
-  <si>
-    <t>10698467</t>
-  </si>
-  <si>
-    <t>BelgiumTen</t>
-  </si>
-  <si>
-    <t>Retail Assistant Cash Office_NEW</t>
-  </si>
-  <si>
-    <t>258 Cash Office</t>
-  </si>
-  <si>
-    <t>Belgium Category III - Experience 10</t>
-  </si>
-  <si>
-    <t>CAT III 3 Year Seniority</t>
-  </si>
-  <si>
-    <t>Test11</t>
-  </si>
-  <si>
-    <t>10698468</t>
-  </si>
-  <si>
-    <t>BelgiumEleven</t>
-  </si>
-  <si>
-    <t>Supervisor_NEW</t>
-  </si>
-  <si>
-    <t>253 Supervisors</t>
-  </si>
-  <si>
-    <t>Variable | 28 | A28</t>
-  </si>
-  <si>
-    <t>Test12</t>
-  </si>
-  <si>
-    <t>10698469</t>
-  </si>
-  <si>
-    <t>BelgiumTweleve</t>
-  </si>
-  <si>
-    <t>Visual Merchandiser_NEW</t>
-  </si>
-  <si>
-    <t>256 Visual Merchandising</t>
-  </si>
-  <si>
-    <t>Belgium Retail - Visual Merchandiser - Experience 1</t>
-  </si>
-  <si>
-    <t>CAT III 1 Year Seniority</t>
-  </si>
-  <si>
-    <t>Test13</t>
-  </si>
-  <si>
-    <t>10698470</t>
-  </si>
-  <si>
-    <t>BelgiumThirteen</t>
-  </si>
-  <si>
-    <t>Supervisor Stockroom_NEW</t>
-  </si>
-  <si>
-    <t>255 Stockroom</t>
-  </si>
-  <si>
-    <t>Variable | 20 | A20/4</t>
-  </si>
-  <si>
-    <t>Test14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test failed for 'BelgiumFourteen TwentyFiveJuneNine' Employee:{Mupol Bypitu }TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for locator('text=Onboarding Guide: In-Store P&amp;C Assistant_NEW - BelgiumFourteen TwentyFiveJuneNine')[22m
-</t>
-  </si>
-  <si>
     <t>BelgiumFourteen</t>
   </si>
   <si>
@@ -651,10 +682,13 @@
     <t>Test15</t>
   </si>
   <si>
+    <t>10698611</t>
+  </si>
+  <si>
     <t>BelgiumFifteen</t>
   </si>
   <si>
-    <t>Auto 26294116</t>
+    <t>Auto 56123073</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -731,7 +765,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -872,7 +906,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -992,6 +1026,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1273,7 +1311,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BQ16"/>
+  <dimension ref="A1:BR17"/>
   <sheetFormatPr defaultRowHeight="15.6" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="10.77734375" style="1" customWidth="1"/>
@@ -1282,7 +1320,7 @@
     <col min="5" max="5" width="7.44140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="5.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="13" style="1" customWidth="1"/>
     <col min="10" max="10" width="11.5546875" style="1" customWidth="1"/>
     <col min="11" max="11" width="5.77734375" style="1" customWidth="1"/>
@@ -1307,7 +1345,7 @@
     <col min="30" max="30" width="11.44140625" style="1" customWidth="1"/>
     <col min="31" max="31" width="20.6640625" style="1" customWidth="1"/>
     <col min="32" max="32" width="31.109375" style="1" customWidth="1"/>
-    <col min="33" max="33" width="14.77734375" style="1" customWidth="1"/>
+    <col min="33" max="33" width="9.21875" style="1" customWidth="1"/>
     <col min="34" max="34" width="18.6640625" style="1" customWidth="1"/>
     <col min="35" max="35" width="26.77734375" style="1" customWidth="1"/>
     <col min="36" max="36" width="16.6640625" style="1" customWidth="1"/>
@@ -1342,9 +1380,10 @@
     <col min="67" max="67" width="17.109375" style="1" customWidth="1"/>
     <col min="68" max="68" width="16.5546875" style="1" customWidth="1"/>
     <col min="69" max="69" width="16.109375" customWidth="1"/>
+    <col min="70" max="70" width="27.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" s="3" customFormat="1" ht="14.55" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:70" s="3" customFormat="1" ht="14.55" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1552,50 +1591,53 @@
       <c r="BQ1" s="7" t="s">
         <v>65</v>
       </c>
+      <c r="BR1" s="7" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="2" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I2" s="18">
         <v>25041111</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L2" s="19">
         <f t="shared" ref="L2:L16" ca="1" si="0">TODAY()-31</f>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O2" s="18">
         <v>38</v>
@@ -1604,44 +1646,44 @@
         <v>1000</v>
       </c>
       <c r="Q2" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R2" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S2" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T2" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U2" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V2" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W2" s="22">
         <f t="shared" ref="W2:W16" ca="1" si="1">L2</f>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X2" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y2" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z2" s="24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA2" s="25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AB2" s="24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC2" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD2" s="24" t="s">
         <v>52</v>
@@ -1650,165 +1692,168 @@
         <v>35</v>
       </c>
       <c r="AF2" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG2" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH2" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI2" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ2" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK2" s="24" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AL2" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM2" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN2" s="1">
         <f t="array" aca="1" ref="AN2" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>68862601559</v>
+        <v>58677936581</v>
       </c>
       <c r="AO2" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP2" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ2" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR2" s="19" t="str">
         <f t="shared" ref="AR2:AR16" si="2">AH2</f>
         <v>N/A</v>
       </c>
       <c r="AS2" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT2" s="28">
         <v>35591</v>
       </c>
       <c r="AU2" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV2" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW2" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW2" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX2" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY2" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ2" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA2" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB2" s="24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="BC2" s="24" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="BD2" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE2" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF2" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG2" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH2" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI2" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ2" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK2" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL2" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM2" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN2" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO2" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP2" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ2" s="33">
         <v>100</v>
       </c>
+      <c r="BR2" s="29" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="3" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B3" s="11">
-        <v>10698459</v>
+        <v>118</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>119</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>121</v>
+        <v>74</v>
       </c>
       <c r="I3" s="18">
         <v>25041111</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L3" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O3" s="18">
         <v>38</v>
@@ -1817,44 +1862,44 @@
         <v>1000</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S3" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T3" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U3" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V3" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W3" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X3" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y3" s="23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Z3" s="24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AA3" s="25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AB3" s="24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC3" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD3" s="24" t="s">
         <v>52</v>
@@ -1863,166 +1908,169 @@
         <v>35</v>
       </c>
       <c r="AF3" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG3" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH3" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AI3" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ3" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK3" s="24">
         <v>251</v>
       </c>
       <c r="AL3" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM3" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN3" s="1">
         <f t="array" aca="1" ref="AN3" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>93994314052</v>
+        <v>69159552547</v>
       </c>
       <c r="AO3" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP3" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AQ3" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR3" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AS3" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AT3" s="28">
         <v>35591</v>
       </c>
       <c r="AU3" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV3" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW3" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW3" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX3" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY3" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ3" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA3" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB3" s="34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="BC3" s="24" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BD3" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE3" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF3" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG3" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH3" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI3" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ3" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK3" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL3" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM3" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN3" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO3" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP3" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ3" s="33">
         <v>100</v>
       </c>
+      <c r="BR3" s="29" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="4" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="11">
-        <v>10698460</v>
+        <v>132</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>133</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I4" s="18">
         <v>25041111</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L4" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O4" s="18">
         <v>38</v>
@@ -2031,44 +2079,44 @@
         <v>1000</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R4" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S4" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T4" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U4" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V4" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W4" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X4" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y4" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z4" s="24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA4" s="25" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="AB4" s="24" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC4" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD4" s="24" t="s">
         <v>52</v>
@@ -2077,165 +2125,168 @@
         <v>20</v>
       </c>
       <c r="AF4" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG4" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH4" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI4" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ4" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK4" s="24" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="AL4" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM4" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN4" s="1">
         <f t="array" aca="1" ref="AN4" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>21779498096</v>
+        <v>35007071680</v>
       </c>
       <c r="AO4" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP4" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ4" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR4" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS4" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT4" s="28">
         <v>35591</v>
       </c>
       <c r="AU4" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV4" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW4" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW4" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX4" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY4" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ4" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA4" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB4" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BC4" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BD4" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE4" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF4" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG4" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH4" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI4" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ4" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK4" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL4" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM4" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN4" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO4" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP4" s="32" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="BQ4" s="33">
         <v>100</v>
       </c>
+      <c r="BR4" s="29" t="s">
+        <v>140</v>
+      </c>
     </row>
-    <row r="5" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B5" s="11">
-        <v>10698461</v>
+        <v>141</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>142</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I5" s="18">
         <v>25041111</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L5" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O5" s="18">
         <v>38</v>
@@ -2244,44 +2295,44 @@
         <v>1000</v>
       </c>
       <c r="Q5" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R5" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S5" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T5" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U5" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V5" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W5" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X5" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y5" s="23" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="Z5" s="24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA5" s="25" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="AB5" s="24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC5" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD5" s="24" t="s">
         <v>52</v>
@@ -2290,165 +2341,168 @@
         <v>35</v>
       </c>
       <c r="AF5" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG5" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH5" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI5" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ5" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK5" s="24">
         <v>251</v>
       </c>
       <c r="AL5" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN5" s="1">
         <f t="array" aca="1" ref="AN5" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>36457753212</v>
+        <v>81247989030</v>
       </c>
       <c r="AO5" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP5" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ5" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR5" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS5" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AT5" s="28">
         <v>35591</v>
       </c>
       <c r="AU5" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV5" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW5" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW5" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX5" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY5" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ5" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA5" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB5" s="34" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="BC5" s="24" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="BD5" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE5" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF5" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG5" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH5" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI5" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ5" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK5" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL5" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM5" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN5" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO5" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP5" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ5" s="33">
         <v>100</v>
       </c>
+      <c r="BR5" s="29" t="s">
+        <v>148</v>
+      </c>
     </row>
-    <row r="6" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I6" s="18">
         <v>25041111</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L6" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O6" s="18">
         <v>38</v>
@@ -2457,44 +2511,44 @@
         <v>1000</v>
       </c>
       <c r="Q6" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R6" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S6" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T6" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U6" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V6" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W6" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X6" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y6" s="35" t="s">
-        <v>82</v>
-      </c>
-      <c r="Z6" s="24" t="s">
-        <v>145</v>
+        <v>83</v>
+      </c>
+      <c r="Z6" s="36" t="s">
+        <v>124</v>
       </c>
       <c r="AA6" s="25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AB6" s="24" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC6" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD6" s="24" t="s">
         <v>52</v>
@@ -2503,166 +2557,169 @@
         <v>30</v>
       </c>
       <c r="AF6" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG6" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH6" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AI6" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ6" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK6" s="24" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="AL6" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN6" s="1">
         <f t="array" aca="1" ref="AN6" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>43444326011</v>
+        <v>28067860541</v>
       </c>
       <c r="AO6" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP6" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AQ6" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR6" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AS6" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT6" s="28">
         <v>35591</v>
       </c>
       <c r="AU6" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV6" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW6" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW6" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX6" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY6" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ6" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA6" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB6" s="24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="BC6" s="24" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="BD6" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE6" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF6" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG6" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH6" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI6" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ6" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK6" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL6" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM6" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN6" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO6" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP6" s="32" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="BQ6" s="33">
         <v>100</v>
       </c>
+      <c r="BR6" s="29" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="7" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B7" s="11">
-        <v>10698463</v>
+        <v>154</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>155</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I7" s="18">
         <v>25041111</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L7" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O7" s="18">
         <v>38</v>
@@ -2671,44 +2728,44 @@
         <v>1000</v>
       </c>
       <c r="Q7" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R7" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S7" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T7" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U7" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V7" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W7" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X7" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y7" s="23" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="Z7" s="36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="AB7" s="37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC7" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD7" s="24" t="s">
         <v>52</v>
@@ -2717,165 +2774,168 @@
         <v>30</v>
       </c>
       <c r="AF7" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG7" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH7" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI7" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ7" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK7" s="24">
         <v>251</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN7" s="1">
         <f t="array" aca="1" ref="AN7" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>29197137746</v>
+        <v>88227162137</v>
       </c>
       <c r="AO7" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP7" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ7" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR7" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS7" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT7" s="28">
         <v>35591</v>
       </c>
       <c r="AU7" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV7" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW7" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW7" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX7" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY7" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ7" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA7" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB7" s="24" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="BC7" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="BD7" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="BE7" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF7" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="BG7" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="BH7" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="BI7" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="BJ7" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="BK7" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="BL7" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="BM7" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN7" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BO7" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BP7" s="32" t="s">
         <v>153</v>
-      </c>
-      <c r="BD7" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="BE7" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="BF7" s="31" t="s">
-        <v>105</v>
-      </c>
-      <c r="BG7" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="BH7" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="BI7" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="BJ7" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="BK7" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="BL7" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="BM7" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="BN7" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="BO7" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="BP7" s="32" t="s">
-        <v>147</v>
       </c>
       <c r="BQ7" s="33">
         <v>100</v>
       </c>
+      <c r="BR7" s="29" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="8" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B8" s="11">
-        <v>10698464</v>
+        <v>161</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>121</v>
+        <v>74</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L8" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O8" s="18">
         <v>38</v>
@@ -2884,44 +2944,44 @@
         <v>1000</v>
       </c>
       <c r="Q8" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R8" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S8" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T8" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U8" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V8" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W8" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X8" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y8" s="23" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="Z8" s="36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="AB8" s="37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC8" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD8" s="24" t="s">
         <v>52</v>
@@ -2930,166 +2990,169 @@
         <v>35</v>
       </c>
       <c r="AF8" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG8" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH8" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AI8" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ8" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK8" s="24">
         <v>251</v>
       </c>
       <c r="AL8" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM8" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN8" s="1">
         <f t="array" aca="1" ref="AN8" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>28141011648</v>
+        <v>51067219144</v>
       </c>
       <c r="AO8" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP8" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AQ8" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR8" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AS8" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT8" s="28">
         <v>35591</v>
       </c>
       <c r="AU8" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV8" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW8" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW8" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX8" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY8" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ8" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA8" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB8" s="24" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="BC8" s="24" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="BD8" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE8" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF8" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG8" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH8" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI8" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ8" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK8" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL8" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM8" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN8" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO8" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP8" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ8" s="33">
         <v>100</v>
       </c>
+      <c r="BR8" s="29" t="s">
+        <v>140</v>
+      </c>
     </row>
-    <row r="9" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="B9" s="11">
-        <v>10698465</v>
+        <v>168</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>169</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
       </c>
       <c r="J9" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L9" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O9" s="18">
         <v>38</v>
@@ -3098,44 +3161,44 @@
         <v>1000</v>
       </c>
       <c r="Q9" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R9" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S9" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T9" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U9" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V9" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W9" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X9" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y9" s="23" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="Z9" s="36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="AB9" s="37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC9" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD9" s="24" t="s">
         <v>52</v>
@@ -3144,165 +3207,168 @@
         <v>20</v>
       </c>
       <c r="AF9" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG9" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH9" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI9" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ9" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK9" s="24">
         <v>251</v>
       </c>
       <c r="AL9" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM9" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN9" s="1">
         <f t="array" aca="1" ref="AN9" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>88781270421</v>
+        <v>83199008557</v>
       </c>
       <c r="AO9" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP9" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ9" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR9" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS9" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT9" s="28">
         <v>35591</v>
       </c>
       <c r="AU9" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV9" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW9" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW9" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX9" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY9" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ9" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA9" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB9" s="24" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="BC9" s="24" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="BD9" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE9" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF9" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG9" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH9" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI9" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ9" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK9" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL9" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM9" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN9" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO9" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP9" s="32" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="BQ9" s="33">
         <v>100</v>
       </c>
+      <c r="BR9" s="29" t="s">
+        <v>148</v>
+      </c>
     </row>
-    <row r="10" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
       </c>
       <c r="J10" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L10" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O10" s="18">
         <v>38</v>
@@ -3311,212 +3377,215 @@
         <v>1000</v>
       </c>
       <c r="Q10" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R10" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S10" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T10" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U10" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V10" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W10" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X10" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y10" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="AB10" s="37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC10" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD10" s="24" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
       </c>
       <c r="AF10" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG10" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH10" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AI10" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ10" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK10" s="24" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="AL10" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM10" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN10" s="1">
         <f t="array" aca="1" ref="AN10" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>97580190593</v>
+        <v>95805410402</v>
       </c>
       <c r="AO10" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP10" s="18" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="AQ10" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR10" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AS10" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT10" s="28">
         <v>35591</v>
       </c>
       <c r="AU10" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV10" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW10" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW10" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX10" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY10" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ10" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA10" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB10" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BC10" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BD10" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE10" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF10" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG10" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH10" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI10" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ10" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK10" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL10" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM10" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN10" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO10" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP10" s="32" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="BQ10" s="33">
         <v>100</v>
       </c>
+      <c r="BR10" s="29" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="11" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
       </c>
       <c r="J11" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L11" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O11" s="18">
         <v>38</v>
@@ -3525,44 +3594,44 @@
         <v>1000</v>
       </c>
       <c r="Q11" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R11" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S11" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T11" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U11" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V11" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W11" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X11" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y11" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z11" s="36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="AB11" s="34" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC11" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD11" s="24" t="s">
         <v>52</v>
@@ -3571,165 +3640,168 @@
         <v>35</v>
       </c>
       <c r="AF11" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG11" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH11" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI11" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ11" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK11" s="24" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="AL11" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM11" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN11" s="1">
         <f t="array" aca="1" ref="AN11" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>44661214921</v>
+        <v>94880039068</v>
       </c>
       <c r="AO11" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP11" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ11" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR11" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS11" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT11" s="28">
         <v>35591</v>
       </c>
       <c r="AU11" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV11" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW11" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW11" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX11" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY11" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ11" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA11" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB11" s="24" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="BC11" s="24" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="BD11" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE11" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF11" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG11" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH11" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI11" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ11" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK11" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL11" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM11" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN11" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO11" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP11" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ11" s="33">
         <v>100</v>
       </c>
+      <c r="BR11" s="29" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="12" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
       </c>
       <c r="J12" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K12" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L12" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M12" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O12" s="18">
         <v>38</v>
@@ -3738,44 +3810,44 @@
         <v>1000</v>
       </c>
       <c r="Q12" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R12" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S12" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T12" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U12" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V12" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W12" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X12" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y12" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z12" s="36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="AB12" s="37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC12" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD12" s="24" t="s">
         <v>52</v>
@@ -3784,165 +3856,168 @@
         <v>28</v>
       </c>
       <c r="AF12" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG12" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH12" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI12" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ12" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK12" s="24" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="AL12" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM12" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN12" s="1">
         <f t="array" aca="1" ref="AN12" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>47336777057</v>
+        <v>73727756230</v>
       </c>
       <c r="AO12" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP12" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ12" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR12" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS12" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT12" s="28">
         <v>35591</v>
       </c>
       <c r="AU12" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV12" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW12" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW12" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX12" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY12" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ12" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA12" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB12" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BC12" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BD12" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE12" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF12" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG12" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH12" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI12" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ12" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK12" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL12" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM12" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN12" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO12" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP12" s="32" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="BQ12" s="33">
         <v>100</v>
       </c>
+      <c r="BR12" s="29" t="s">
+        <v>140</v>
+      </c>
     </row>
-    <row r="13" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
       </c>
       <c r="J13" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K13" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L13" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O13" s="18">
         <v>38</v>
@@ -3951,44 +4026,44 @@
         <v>1000</v>
       </c>
       <c r="Q13" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R13" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S13" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T13" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U13" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V13" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W13" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X13" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y13" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z13" s="36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="AB13" s="37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC13" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD13" s="24" t="s">
         <v>52</v>
@@ -3997,166 +4072,169 @@
         <v>35</v>
       </c>
       <c r="AF13" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG13" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH13" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AI13" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ13" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK13" s="24" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="AL13" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM13" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN13" s="1">
         <f t="array" aca="1" ref="AN13" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>28957789980</v>
+        <v>38491273349</v>
       </c>
       <c r="AO13" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP13" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AQ13" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR13" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AS13" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT13" s="28">
         <v>35591</v>
       </c>
       <c r="AU13" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV13" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW13" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW13" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX13" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY13" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ13" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA13" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB13" s="24" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="BD13" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE13" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF13" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG13" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH13" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI13" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ13" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK13" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL13" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM13" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN13" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO13" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP13" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ13" s="33">
         <v>100</v>
       </c>
+      <c r="BR13" s="29" t="s">
+        <v>148</v>
+      </c>
     </row>
-    <row r="14" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
       </c>
       <c r="J14" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L14" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M14" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O14" s="18">
         <v>38</v>
@@ -4165,44 +4243,44 @@
         <v>1000</v>
       </c>
       <c r="Q14" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R14" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S14" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T14" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U14" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V14" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W14" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X14" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y14" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z14" s="36" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="AB14" s="37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC14" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD14" s="24" t="s">
         <v>52</v>
@@ -4211,165 +4289,168 @@
         <v>20</v>
       </c>
       <c r="AF14" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG14" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH14" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI14" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ14" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK14" s="34" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="AL14" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM14" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN14" s="1">
         <f t="array" aca="1" ref="AN14" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>51349978822</v>
+        <v>22939868167</v>
       </c>
       <c r="AO14" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP14" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ14" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR14" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS14" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT14" s="28">
         <v>35591</v>
       </c>
       <c r="AU14" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV14" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW14" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW14" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX14" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY14" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ14" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA14" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB14" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BC14" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BD14" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE14" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF14" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG14" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH14" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI14" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ14" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK14" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL14" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM14" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN14" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO14" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP14" s="32" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="BQ14" s="33">
         <v>100</v>
       </c>
+      <c r="BR14" s="29" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="15" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>117</v>
+        <v>211</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
       </c>
       <c r="J15" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K15" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L15" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O15" s="18">
         <v>38</v>
@@ -4378,44 +4459,44 @@
         <v>1000</v>
       </c>
       <c r="Q15" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R15" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S15" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T15" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U15" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V15" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W15" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X15" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y15" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z15" s="36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AA15" s="25" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="AB15" s="37" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AC15" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD15" s="24" t="s">
         <v>52</v>
@@ -4424,166 +4505,169 @@
         <v>30</v>
       </c>
       <c r="AF15" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG15" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH15" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AI15" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ15" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AK15" s="24" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="AL15" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM15" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN15" s="1">
         <f t="array" aca="1" ref="AN15" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>98582859372</v>
+        <v>63222815676</v>
       </c>
       <c r="AO15" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP15" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AQ15" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR15" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46183</v>
+        <v>46196</v>
       </c>
       <c r="AS15" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT15" s="28">
         <v>35591</v>
       </c>
       <c r="AU15" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV15" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW15" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW15" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX15" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY15" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ15" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA15" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB15" s="24" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="BC15" s="24" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="BD15" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE15" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF15" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG15" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH15" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI15" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ15" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK15" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL15" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM15" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN15" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO15" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP15" s="32" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="BQ15" s="33">
         <v>100</v>
       </c>
+      <c r="BR15" s="29" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="16" spans="1:69" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B16" s="11">
-        <v>10698471</v>
+        <v>215</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>216</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
       </c>
       <c r="J16" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K16" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L16" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O16" s="18">
         <v>38</v>
@@ -4592,44 +4676,44 @@
         <v>1000</v>
       </c>
       <c r="Q16" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R16" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S16" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="T16" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U16" s="21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="V16" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W16" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45787</v>
+        <v>45800</v>
       </c>
       <c r="X16" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y16" s="23" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="Z16" s="34" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="AB16" s="37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AC16" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AD16" s="24" t="s">
         <v>52</v>
@@ -4638,121 +4722,127 @@
         <v>35</v>
       </c>
       <c r="AF16" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AG16" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AH16" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AI16" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AJ16" s="18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK16" s="24">
         <v>251</v>
       </c>
       <c r="AL16" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AM16" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AN16" s="1">
         <f t="array" aca="1" ref="AN16" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>53875782183</v>
+        <v>64382457098</v>
       </c>
       <c r="AO16" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AP16" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AQ16" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AR16" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS16" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AT16" s="28">
         <v>35591</v>
       </c>
       <c r="AU16" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AV16" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="AW16" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="AW16" s="29" t="s">
-        <v>77</v>
-      </c>
       <c r="AX16" s="29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AY16" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AZ16" s="29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BA16" s="29" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="BB16" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BC16" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="BD16" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BE16" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BF16" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BG16" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BH16" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BI16" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BJ16" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BK16" s="29" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BL16" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BM16" s="29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BN16" s="29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="BO16" s="29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BP16" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BQ16" s="33">
         <v>100</v>
       </c>
+      <c r="BR16" s="29" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="70:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BR17" s="38"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -4781,7 +4871,7 @@
     <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId16"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Termination of Poland & Belgium is completed 1st Aug'25
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Belgium_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Belgium_Regression_PK14.xlsx
@@ -3,15 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{71F158FF-A586-4CED-8B17-1F1FD1529E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD86074-4BF3-4C44-A463-D0498F998D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="221">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -229,13 +228,16 @@
     <t>AllowanceAmount</t>
   </si>
   <si>
+    <t>EducationLevel</t>
+  </si>
+  <si>
     <t>Test1</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'BelgiumOne TwentyFiveJuneNineA' Employee:{undefined}TimeoutError: locator.focus: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for getByLabel('Supervisory Organization')[22m
-</t>
+    <t>10698973</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
   <si>
     <t>751 Retail Team 1 (Mupol Bypitu (10528834) (Inherited))</t>
@@ -250,7 +252,7 @@
     <t>BelgiumOne</t>
   </si>
   <si>
-    <t>TwentyFiveJuneNineA</t>
+    <t>TwentyFiveJulyTwentyEight</t>
   </si>
   <si>
     <t>Landline</t>
@@ -295,7 +297,7 @@
     <t>V2 BIS - (Job Qualifications-Belgium)</t>
   </si>
   <si>
-    <t>5 Days (Belgium)</t>
+    <t>5 Days</t>
   </si>
   <si>
     <t>N/A</t>
@@ -379,10 +381,13 @@
     <t>Variable | 35 | A35</t>
   </si>
   <si>
+    <t>Primary School</t>
+  </si>
+  <si>
     <t>Test2</t>
   </si>
   <si>
-    <t>Test failed for 'BelgiumTwo TwentyFiveJuneNine' Employee:{}Error: page.waitForTimeout: Test ended.</t>
+    <t>10698974</t>
   </si>
   <si>
     <t>751 Store Management (Mupol Bypitu (10528834))</t>
@@ -394,10 +399,7 @@
     <t>BelgiumTwo</t>
   </si>
   <si>
-    <t>TwentyFiveJuneNine</t>
-  </si>
-  <si>
-    <t>Auto 66285002</t>
+    <t>Auto 74502567</t>
   </si>
   <si>
     <t>Fixed Term</t>
@@ -421,10 +423,13 @@
     <t xml:space="preserve">Store Manager - First Store </t>
   </si>
   <si>
+    <t>Secondary School</t>
+  </si>
+  <si>
     <t>Test3</t>
   </si>
   <si>
-    <t>Passed</t>
+    <t>10698975</t>
   </si>
   <si>
     <t>BelgiumThree</t>
@@ -442,13 +447,19 @@
     <t>Variable | 20 | A20</t>
   </si>
   <si>
+    <t>Non-university Higher Education</t>
+  </si>
+  <si>
     <t>Test4</t>
   </si>
   <si>
+    <t>10698976</t>
+  </si>
+  <si>
     <t>BelgiumFour</t>
   </si>
   <si>
-    <t>Auto 28143044</t>
+    <t>Auto 37728090</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -460,10 +471,13 @@
     <t>Team Manager</t>
   </si>
   <si>
+    <t>University</t>
+  </si>
+  <si>
     <t>Test5</t>
   </si>
   <si>
-    <t>10698462</t>
+    <t>10698977</t>
   </si>
   <si>
     <t>BelgiumFive</t>
@@ -481,10 +495,13 @@
     <t>Test6</t>
   </si>
   <si>
+    <t>10698978</t>
+  </si>
+  <si>
     <t>BelgiumSix</t>
   </si>
   <si>
-    <t>Auto 21896146</t>
+    <t>Auto 73972672</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -499,10 +516,13 @@
     <t>Test7</t>
   </si>
   <si>
+    <t>10698979</t>
+  </si>
+  <si>
     <t>BelgiumSeven</t>
   </si>
   <si>
-    <t>Auto 49758543</t>
+    <t>Auto 47073662</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -517,10 +537,13 @@
     <t>Test8</t>
   </si>
   <si>
+    <t>10698980</t>
+  </si>
+  <si>
     <t>BelgiumEight</t>
   </si>
   <si>
-    <t>Auto 48512271</t>
+    <t>Auto 28112732</t>
   </si>
   <si>
     <t>Visual Merchandising Manager_NEW</t>
@@ -535,10 +558,10 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10698466</t>
-  </si>
-  <si>
-    <t>BelgiumNineReRun</t>
+    <t>10698981</t>
+  </si>
+  <si>
+    <t>BelgiumNine</t>
   </si>
   <si>
     <t>Students</t>
@@ -559,7 +582,7 @@
     <t>Test10</t>
   </si>
   <si>
-    <t>10698467</t>
+    <t>10698982</t>
   </si>
   <si>
     <t>BelgiumTen</t>
@@ -580,7 +603,7 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10698468</t>
+    <t>10698983</t>
   </si>
   <si>
     <t>BelgiumEleven</t>
@@ -598,12 +621,15 @@
     <t>Test12</t>
   </si>
   <si>
-    <t>10698469</t>
+    <t>10698987</t>
   </si>
   <si>
     <t>BelgiumTweleve</t>
   </si>
   <si>
+    <t>TwentyFiveJulyTwentyEightA</t>
+  </si>
+  <si>
     <t>Visual Merchandiser_NEW</t>
   </si>
   <si>
@@ -619,7 +645,7 @@
     <t>Test13</t>
   </si>
   <si>
-    <t>10698470</t>
+    <t>10698984</t>
   </si>
   <si>
     <t>BelgiumThirteen</t>
@@ -637,15 +663,15 @@
     <t>Test14</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'BelgiumFourteen TwentyFiveJuneNine' Employee:{Mupol Bypitu }TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for locator('text=Onboarding Guide: In-Store P&amp;C Assistant_NEW - BelgiumFourteen TwentyFiveJuneNine')[22m
-</t>
+    <t>10699011</t>
   </si>
   <si>
     <t>BelgiumFourteen</t>
   </si>
   <si>
+    <t>TwentyFiveJulyTwentyEightB</t>
+  </si>
+  <si>
     <t>Belgium Retail - P&amp;C Assistant (entry, 1st increase, good experience)</t>
   </si>
   <si>
@@ -655,10 +681,13 @@
     <t>Test15</t>
   </si>
   <si>
+    <t>10698986</t>
+  </si>
+  <si>
     <t>BelgiumFifteen</t>
   </si>
   <si>
-    <t>Auto 26294116</t>
+    <t>Auto 45711605</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -735,7 +764,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -1277,78 +1306,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BQ16"/>
-  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BR16"/>
+  <sheetFormatPr defaultRowHeight="15.6" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="48.1796875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.453125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="5.54296875" style="1" customWidth="1"/>
+    <col min="1" max="2" width="10.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="48.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="5.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" style="1" customWidth="1"/>
     <col min="9" max="9" width="13" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="5.81640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.81640625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="7.453125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.81640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="5.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.77734375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="7.44140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.77734375" style="2" customWidth="1"/>
     <col min="15" max="15" width="13" style="1" customWidth="1"/>
-    <col min="16" max="16" width="10.08984375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="7.6328125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="20.1796875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="5.81640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="10.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="7.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="20.21875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="5.77734375" style="1" customWidth="1"/>
     <col min="20" max="20" width="13" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.81640625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="5.81640625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="12.1796875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.453125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="19.90625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="13.08984375" style="2" customWidth="1"/>
-    <col min="27" max="27" width="18.6328125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="8.90625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="8.453125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="11.453125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="20.6328125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="31.08984375" style="1" customWidth="1"/>
-    <col min="33" max="33" width="14.81640625" style="1" customWidth="1"/>
-    <col min="34" max="34" width="18.6328125" style="1" customWidth="1"/>
-    <col min="35" max="35" width="26.81640625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="16.6328125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="17.08984375" style="1" customWidth="1"/>
-    <col min="38" max="38" width="20.453125" style="1" customWidth="1"/>
-    <col min="39" max="40" width="22.453125" style="1" customWidth="1"/>
-    <col min="41" max="41" width="18.1796875" style="1" customWidth="1"/>
-    <col min="42" max="42" width="17.81640625" style="1" customWidth="1"/>
-    <col min="43" max="43" width="5.90625" style="1" customWidth="1"/>
-    <col min="44" max="44" width="15.08984375" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="5.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="12.21875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.44140625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="19.88671875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="13.109375" style="2" customWidth="1"/>
+    <col min="27" max="27" width="18.6640625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="8.88671875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="8.44140625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="11.44140625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="20.6640625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="31.109375" style="1" customWidth="1"/>
+    <col min="33" max="33" width="14.77734375" style="1" customWidth="1"/>
+    <col min="34" max="34" width="18.6640625" style="1" customWidth="1"/>
+    <col min="35" max="35" width="26.77734375" style="1" customWidth="1"/>
+    <col min="36" max="36" width="16.6640625" style="1" customWidth="1"/>
+    <col min="37" max="37" width="17.109375" style="1" customWidth="1"/>
+    <col min="38" max="38" width="20.44140625" style="1" customWidth="1"/>
+    <col min="39" max="40" width="22.44140625" style="1" customWidth="1"/>
+    <col min="41" max="41" width="18.21875" style="1" customWidth="1"/>
+    <col min="42" max="42" width="17.77734375" style="1" customWidth="1"/>
+    <col min="43" max="43" width="5.88671875" style="1" customWidth="1"/>
+    <col min="44" max="44" width="15.109375" style="1" customWidth="1"/>
     <col min="45" max="45" width="7" style="1" customWidth="1"/>
-    <col min="46" max="46" width="10.81640625" style="1" customWidth="1"/>
-    <col min="47" max="47" width="13.54296875" style="1" customWidth="1"/>
-    <col min="48" max="48" width="20.1796875" style="1" customWidth="1"/>
-    <col min="49" max="49" width="9.90625" style="1" customWidth="1"/>
-    <col min="50" max="50" width="11.90625" style="1" customWidth="1"/>
-    <col min="51" max="51" width="15.90625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="10.77734375" style="1" customWidth="1"/>
+    <col min="47" max="47" width="13.5546875" style="1" customWidth="1"/>
+    <col min="48" max="48" width="20.21875" style="1" customWidth="1"/>
+    <col min="49" max="49" width="9.88671875" style="1" customWidth="1"/>
+    <col min="50" max="50" width="11.88671875" style="1" customWidth="1"/>
+    <col min="51" max="51" width="15.88671875" style="1" customWidth="1"/>
     <col min="52" max="52" width="15" style="1" customWidth="1"/>
-    <col min="53" max="53" width="16.36328125" style="2" customWidth="1"/>
-    <col min="54" max="54" width="53.6328125" style="2" customWidth="1"/>
-    <col min="55" max="55" width="23.81640625" style="2" customWidth="1"/>
+    <col min="53" max="53" width="16.33203125" style="2" customWidth="1"/>
+    <col min="54" max="54" width="53.6640625" style="2" customWidth="1"/>
+    <col min="55" max="55" width="23.77734375" style="2" customWidth="1"/>
     <col min="56" max="56" width="9" style="1" customWidth="1"/>
-    <col min="57" max="57" width="30.08984375" style="1" customWidth="1"/>
-    <col min="58" max="58" width="20.36328125" style="1" customWidth="1"/>
-    <col min="59" max="59" width="14.453125" style="1" customWidth="1"/>
-    <col min="60" max="60" width="17.08984375" style="1" customWidth="1"/>
-    <col min="61" max="61" width="11.54296875" style="1" customWidth="1"/>
-    <col min="62" max="62" width="15.453125" style="1" customWidth="1"/>
-    <col min="63" max="64" width="11.08984375" style="1" customWidth="1"/>
-    <col min="65" max="65" width="16.6328125" style="1" customWidth="1"/>
-    <col min="66" max="66" width="18.08984375" style="1" customWidth="1"/>
-    <col min="67" max="67" width="17.08984375" style="1" customWidth="1"/>
-    <col min="68" max="68" width="16.54296875" style="1" customWidth="1"/>
-    <col min="69" max="69" width="16.08984375" customWidth="1"/>
+    <col min="57" max="57" width="30.109375" style="1" customWidth="1"/>
+    <col min="58" max="58" width="20.33203125" style="1" customWidth="1"/>
+    <col min="59" max="59" width="14.44140625" style="1" customWidth="1"/>
+    <col min="60" max="60" width="17.109375" style="1" customWidth="1"/>
+    <col min="61" max="61" width="11.5546875" style="1" customWidth="1"/>
+    <col min="62" max="62" width="15.44140625" style="1" customWidth="1"/>
+    <col min="63" max="64" width="11.109375" style="1" customWidth="1"/>
+    <col min="65" max="65" width="16.6640625" style="1" customWidth="1"/>
+    <col min="66" max="66" width="18.109375" style="1" customWidth="1"/>
+    <col min="67" max="67" width="17.109375" style="1" customWidth="1"/>
+    <col min="68" max="68" width="16.5546875" style="1" customWidth="1"/>
+    <col min="69" max="69" width="16.109375" customWidth="1"/>
+    <col min="70" max="70" width="27.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:70" s="3" customFormat="1" ht="14.55" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1556,50 +1586,53 @@
       <c r="BQ1" s="7" t="s">
         <v>65</v>
       </c>
+      <c r="BR1" s="7" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="2" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I2" s="18">
         <v>25041111</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L2" s="19">
         <f t="shared" ref="L2:L16" ca="1" si="0">TODAY()-31</f>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O2" s="18">
         <v>38</v>
@@ -1608,44 +1641,44 @@
         <v>1000</v>
       </c>
       <c r="Q2" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R2" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S2" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R2" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S2" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T2" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U2" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V2" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W2" s="22">
         <f t="shared" ref="W2:W16" ca="1" si="1">L2</f>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X2" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y2" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z2" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA2" s="25" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AB2" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC2" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD2" s="24" t="s">
         <v>52</v>
@@ -1654,165 +1687,168 @@
         <v>35</v>
       </c>
       <c r="AF2" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG2" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH2" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI2" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ2" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK2" s="24" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AL2" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM2" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN2" s="1">
         <f t="array" aca="1" ref="AN2" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>71719789375</v>
+        <v>38650979416</v>
       </c>
       <c r="AO2" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP2" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ2" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR2" s="19" t="str">
         <f t="shared" ref="AR2:AR16" si="2">AH2</f>
         <v>N/A</v>
       </c>
       <c r="AS2" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT2" s="28">
         <v>35591</v>
       </c>
       <c r="AU2" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV2" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW2" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX2" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY2" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ2" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA2" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB2" s="24" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="BC2" s="24" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="BD2" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE2" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF2" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG2" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH2" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI2" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ2" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK2" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL2" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM2" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN2" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO2" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP2" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ2" s="33">
         <v>100</v>
       </c>
+      <c r="BR2" s="27" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="3" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I3" s="18">
         <v>25041111</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L3" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O3" s="18">
         <v>38</v>
@@ -1821,44 +1857,44 @@
         <v>1000</v>
       </c>
       <c r="Q3" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R3" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R3" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S3" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T3" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U3" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V3" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W3" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X3" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y3" s="23" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="Z3" s="24" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AA3" s="25" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="AB3" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC3" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD3" s="24" t="s">
         <v>52</v>
@@ -1867,166 +1903,169 @@
         <v>35</v>
       </c>
       <c r="AF3" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="AG3" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH3" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AI3" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ3" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AK3" s="24">
         <v>251</v>
       </c>
       <c r="AL3" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM3" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN3" s="1">
         <f t="array" aca="1" ref="AN3" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>91502395066</v>
+        <v>38115971385</v>
       </c>
       <c r="AO3" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP3" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AQ3" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR3" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AS3" s="24" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="AT3" s="28">
         <v>35591</v>
       </c>
       <c r="AU3" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV3" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW3" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX3" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY3" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ3" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA3" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB3" s="34" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="BC3" s="24" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="BD3" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE3" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF3" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG3" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH3" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI3" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ3" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK3" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL3" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM3" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN3" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO3" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP3" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ3" s="33">
         <v>100</v>
       </c>
+      <c r="BR3" s="27" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="4" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B4" s="11">
-        <v>10698460</v>
+        <v>132</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>133</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I4" s="18">
         <v>25041111</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L4" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O4" s="18">
         <v>38</v>
@@ -2035,44 +2074,44 @@
         <v>1000</v>
       </c>
       <c r="Q4" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R4" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S4" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R4" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S4" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T4" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U4" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V4" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W4" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X4" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y4" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z4" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA4" s="25" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AB4" s="24" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC4" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD4" s="24" t="s">
         <v>52</v>
@@ -2081,165 +2120,168 @@
         <v>20</v>
       </c>
       <c r="AF4" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG4" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH4" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI4" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ4" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK4" s="24" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="AL4" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM4" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN4" s="1">
         <f t="array" aca="1" ref="AN4" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>40121488835</v>
+        <v>61201462928</v>
       </c>
       <c r="AO4" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP4" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ4" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR4" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS4" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT4" s="28">
         <v>35591</v>
       </c>
       <c r="AU4" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV4" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW4" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX4" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY4" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ4" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA4" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB4" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BC4" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BD4" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE4" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF4" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG4" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH4" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI4" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ4" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK4" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL4" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM4" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN4" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO4" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP4" s="32" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="BQ4" s="33">
         <v>100</v>
       </c>
+      <c r="BR4" s="27" t="s">
+        <v>139</v>
+      </c>
     </row>
-    <row r="5" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B5" s="11">
-        <v>10698461</v>
+        <v>140</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>141</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I5" s="18">
         <v>25041111</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L5" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O5" s="18">
         <v>38</v>
@@ -2248,44 +2290,44 @@
         <v>1000</v>
       </c>
       <c r="Q5" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R5" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S5" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R5" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S5" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T5" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U5" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V5" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W5" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X5" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y5" s="23" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="Z5" s="24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA5" s="25" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="AB5" s="24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC5" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD5" s="24" t="s">
         <v>52</v>
@@ -2294,165 +2336,168 @@
         <v>35</v>
       </c>
       <c r="AF5" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="AG5" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH5" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI5" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ5" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AK5" s="24">
         <v>251</v>
       </c>
       <c r="AL5" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM5" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN5" s="1">
         <f t="array" aca="1" ref="AN5" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>94947444497</v>
+        <v>41255431304</v>
       </c>
       <c r="AO5" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP5" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ5" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR5" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS5" s="24" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="AT5" s="28">
         <v>35591</v>
       </c>
       <c r="AU5" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV5" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW5" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX5" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY5" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ5" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA5" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB5" s="34" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="BC5" s="24" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="BD5" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE5" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF5" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG5" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH5" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI5" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ5" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK5" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL5" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM5" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN5" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO5" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP5" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ5" s="33">
         <v>100</v>
       </c>
+      <c r="BR5" s="27" t="s">
+        <v>147</v>
+      </c>
     </row>
-    <row r="6" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I6" s="18">
         <v>25041111</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L6" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M6" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O6" s="18">
         <v>38</v>
@@ -2461,44 +2506,44 @@
         <v>1000</v>
       </c>
       <c r="Q6" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R6" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S6" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R6" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S6" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T6" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U6" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V6" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W6" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X6" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y6" s="35" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z6" s="24" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="AA6" s="25" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AB6" s="24" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC6" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD6" s="24" t="s">
         <v>52</v>
@@ -2507,166 +2552,169 @@
         <v>30</v>
       </c>
       <c r="AF6" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG6" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH6" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AI6" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ6" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK6" s="24" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="AL6" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM6" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN6" s="1">
         <f t="array" aca="1" ref="AN6" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>25656057960</v>
+        <v>32935208490</v>
       </c>
       <c r="AO6" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP6" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AQ6" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR6" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AS6" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT6" s="28">
         <v>35591</v>
       </c>
       <c r="AU6" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV6" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW6" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX6" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY6" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ6" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA6" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB6" s="24" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="BC6" s="24" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="BD6" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE6" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF6" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG6" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH6" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI6" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ6" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK6" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL6" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM6" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN6" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO6" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP6" s="32" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="BQ6" s="33">
         <v>100</v>
       </c>
+      <c r="BR6" s="27" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="7" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B7" s="11">
-        <v>10698463</v>
+        <v>154</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>155</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I7" s="18">
         <v>25041111</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L7" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O7" s="18">
         <v>38</v>
@@ -2675,44 +2723,44 @@
         <v>1000</v>
       </c>
       <c r="Q7" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R7" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S7" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R7" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S7" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T7" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U7" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V7" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W7" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X7" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y7" s="23" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="Z7" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="AB7" s="37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC7" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD7" s="24" t="s">
         <v>52</v>
@@ -2721,165 +2769,168 @@
         <v>30</v>
       </c>
       <c r="AF7" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG7" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH7" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI7" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ7" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AK7" s="24">
         <v>251</v>
       </c>
       <c r="AL7" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM7" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN7" s="1">
         <f t="array" aca="1" ref="AN7" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>82079222230</v>
+        <v>86384924252</v>
       </c>
       <c r="AO7" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP7" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ7" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR7" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS7" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT7" s="28">
         <v>35591</v>
       </c>
       <c r="AU7" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV7" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW7" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX7" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY7" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ7" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA7" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB7" s="24" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="BC7" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="BD7" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="BE7" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF7" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="BG7" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="BH7" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="BI7" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="BJ7" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="BK7" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="BL7" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="BM7" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN7" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BO7" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BP7" s="32" t="s">
         <v>153</v>
-      </c>
-      <c r="BD7" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="BE7" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="BF7" s="31" t="s">
-        <v>104</v>
-      </c>
-      <c r="BG7" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="BH7" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="BI7" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="BJ7" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="BK7" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="BL7" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="BM7" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="BN7" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="BO7" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="BP7" s="32" t="s">
-        <v>147</v>
       </c>
       <c r="BQ7" s="33">
         <v>100</v>
       </c>
+      <c r="BR7" s="27" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="8" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B8" s="11">
-        <v>10698464</v>
+        <v>161</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L8" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O8" s="18">
         <v>38</v>
@@ -2888,44 +2939,44 @@
         <v>1000</v>
       </c>
       <c r="Q8" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R8" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S8" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R8" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S8" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T8" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U8" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V8" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W8" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X8" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y8" s="23" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="Z8" s="36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="AB8" s="37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC8" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD8" s="24" t="s">
         <v>52</v>
@@ -2934,166 +2985,169 @@
         <v>35</v>
       </c>
       <c r="AF8" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG8" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH8" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AI8" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ8" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AK8" s="24">
         <v>251</v>
       </c>
       <c r="AL8" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM8" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN8" s="1">
         <f t="array" aca="1" ref="AN8" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>28542579758</v>
+        <v>86685327614</v>
       </c>
       <c r="AO8" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP8" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AQ8" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR8" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AS8" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT8" s="28">
         <v>35591</v>
       </c>
       <c r="AU8" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV8" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW8" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX8" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY8" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ8" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA8" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB8" s="24" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="BC8" s="24" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="BD8" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE8" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF8" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG8" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH8" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI8" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ8" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK8" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL8" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM8" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN8" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO8" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP8" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ8" s="33">
         <v>100</v>
       </c>
+      <c r="BR8" s="27" t="s">
+        <v>139</v>
+      </c>
     </row>
-    <row r="9" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="B9" s="11">
-        <v>10698465</v>
+        <v>168</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>169</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
       </c>
       <c r="J9" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L9" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O9" s="18">
         <v>38</v>
@@ -3102,44 +3156,44 @@
         <v>1000</v>
       </c>
       <c r="Q9" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R9" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R9" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S9" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T9" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U9" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V9" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W9" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X9" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y9" s="23" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="Z9" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="AB9" s="37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC9" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD9" s="24" t="s">
         <v>52</v>
@@ -3148,165 +3202,168 @@
         <v>20</v>
       </c>
       <c r="AF9" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG9" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH9" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI9" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ9" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AK9" s="24">
         <v>251</v>
       </c>
       <c r="AL9" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM9" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN9" s="1">
         <f t="array" aca="1" ref="AN9" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>72668665926</v>
+        <v>78832823836</v>
       </c>
       <c r="AO9" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP9" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ9" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR9" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS9" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT9" s="28">
         <v>35591</v>
       </c>
       <c r="AU9" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV9" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW9" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX9" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY9" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ9" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA9" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB9" s="24" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="BC9" s="24" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="BD9" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE9" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF9" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG9" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH9" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI9" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ9" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK9" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL9" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM9" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN9" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO9" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP9" s="32" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="BQ9" s="33">
         <v>100</v>
       </c>
+      <c r="BR9" s="27" t="s">
+        <v>147</v>
+      </c>
     </row>
-    <row r="10" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
       </c>
       <c r="J10" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L10" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O10" s="18">
         <v>38</v>
@@ -3315,212 +3372,215 @@
         <v>1000</v>
       </c>
       <c r="Q10" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R10" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S10" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R10" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S10" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T10" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U10" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V10" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W10" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X10" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y10" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="AB10" s="37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC10" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD10" s="24" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
       </c>
       <c r="AF10" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG10" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH10" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AI10" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ10" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK10" s="24" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="AL10" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM10" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN10" s="1">
         <f t="array" aca="1" ref="AN10" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>18751346803</v>
+        <v>45890571389</v>
       </c>
       <c r="AO10" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP10" s="18" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="AQ10" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR10" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AS10" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT10" s="28">
         <v>35591</v>
       </c>
       <c r="AU10" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV10" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW10" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX10" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY10" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ10" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA10" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB10" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BC10" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BD10" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE10" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF10" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG10" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH10" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI10" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ10" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK10" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL10" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM10" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN10" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO10" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP10" s="32" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="BQ10" s="33">
         <v>100</v>
       </c>
+      <c r="BR10" s="27" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="11" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
       </c>
       <c r="J11" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L11" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O11" s="18">
         <v>38</v>
@@ -3529,44 +3589,44 @@
         <v>1000</v>
       </c>
       <c r="Q11" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R11" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S11" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R11" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S11" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T11" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U11" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V11" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W11" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X11" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y11" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z11" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="AB11" s="34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC11" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD11" s="24" t="s">
         <v>52</v>
@@ -3575,165 +3635,168 @@
         <v>35</v>
       </c>
       <c r="AF11" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG11" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH11" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI11" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ11" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK11" s="24" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="AL11" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM11" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN11" s="1">
         <f t="array" aca="1" ref="AN11" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>28433491282</v>
+        <v>78496585364</v>
       </c>
       <c r="AO11" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP11" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ11" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR11" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS11" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT11" s="28">
         <v>35591</v>
       </c>
       <c r="AU11" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV11" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW11" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX11" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY11" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ11" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA11" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB11" s="24" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="BC11" s="24" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="BD11" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE11" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF11" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG11" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH11" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI11" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ11" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK11" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL11" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM11" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN11" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO11" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP11" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ11" s="33">
         <v>100</v>
       </c>
+      <c r="BR11" s="27" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="12" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
       </c>
       <c r="J12" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K12" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L12" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M12" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O12" s="18">
         <v>38</v>
@@ -3742,44 +3805,44 @@
         <v>1000</v>
       </c>
       <c r="Q12" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R12" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S12" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R12" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S12" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T12" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U12" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V12" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W12" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X12" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y12" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z12" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="AB12" s="37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC12" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD12" s="24" t="s">
         <v>52</v>
@@ -3788,165 +3851,168 @@
         <v>28</v>
       </c>
       <c r="AF12" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG12" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH12" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI12" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ12" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK12" s="24" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="AL12" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM12" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN12" s="1">
         <f t="array" aca="1" ref="AN12" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>90571246703</v>
+        <v>28081372603</v>
       </c>
       <c r="AO12" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP12" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ12" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR12" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS12" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT12" s="28">
         <v>35591</v>
       </c>
       <c r="AU12" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV12" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW12" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX12" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY12" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ12" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA12" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB12" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BC12" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BD12" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE12" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF12" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG12" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH12" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI12" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ12" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK12" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL12" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM12" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN12" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO12" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP12" s="32" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="BQ12" s="33">
         <v>100</v>
       </c>
+      <c r="BR12" s="27" t="s">
+        <v>139</v>
+      </c>
     </row>
-    <row r="13" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>120</v>
+        <v>199</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
       </c>
       <c r="J13" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K13" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L13" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O13" s="18">
         <v>38</v>
@@ -3955,44 +4021,44 @@
         <v>1000</v>
       </c>
       <c r="Q13" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R13" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S13" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R13" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S13" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T13" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U13" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V13" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W13" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X13" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y13" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z13" s="36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="AB13" s="37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC13" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD13" s="24" t="s">
         <v>52</v>
@@ -4001,166 +4067,169 @@
         <v>35</v>
       </c>
       <c r="AF13" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG13" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH13" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AI13" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ13" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK13" s="24" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="AL13" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM13" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN13" s="1">
         <f t="array" aca="1" ref="AN13" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>54380828914</v>
+        <v>63825681696</v>
       </c>
       <c r="AO13" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP13" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AQ13" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR13" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AS13" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT13" s="28">
         <v>35591</v>
       </c>
       <c r="AU13" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV13" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW13" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX13" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY13" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ13" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA13" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB13" s="24" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="BD13" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE13" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF13" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG13" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH13" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI13" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ13" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK13" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL13" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM13" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN13" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO13" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP13" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ13" s="33">
         <v>100</v>
       </c>
+      <c r="BR13" s="27" t="s">
+        <v>147</v>
+      </c>
     </row>
-    <row r="14" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
       </c>
       <c r="J14" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L14" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M14" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O14" s="18">
         <v>38</v>
@@ -4169,44 +4238,44 @@
         <v>1000</v>
       </c>
       <c r="Q14" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R14" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S14" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R14" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S14" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T14" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U14" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V14" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W14" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X14" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y14" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z14" s="36" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="AB14" s="37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC14" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD14" s="24" t="s">
         <v>52</v>
@@ -4215,165 +4284,168 @@
         <v>20</v>
       </c>
       <c r="AF14" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG14" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH14" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI14" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ14" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK14" s="34" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="AL14" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM14" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN14" s="1">
         <f t="array" aca="1" ref="AN14" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>69681392868</v>
+        <v>61764971273</v>
       </c>
       <c r="AO14" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP14" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ14" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR14" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS14" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT14" s="28">
         <v>35591</v>
       </c>
       <c r="AU14" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV14" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW14" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX14" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY14" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ14" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA14" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB14" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BC14" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BD14" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE14" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF14" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG14" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH14" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI14" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ14" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK14" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL14" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM14" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN14" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO14" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP14" s="32" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="BQ14" s="33">
         <v>100</v>
       </c>
+      <c r="BR14" s="27" t="s">
+        <v>117</v>
+      </c>
     </row>
-    <row r="15" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>120</v>
+        <v>213</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
       </c>
       <c r="J15" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K15" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L15" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O15" s="18">
         <v>38</v>
@@ -4382,44 +4454,44 @@
         <v>1000</v>
       </c>
       <c r="Q15" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R15" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S15" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R15" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S15" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T15" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U15" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V15" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W15" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X15" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y15" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Z15" s="36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AA15" s="25" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AB15" s="37" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AC15" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD15" s="24" t="s">
         <v>52</v>
@@ -4428,166 +4500,169 @@
         <v>30</v>
       </c>
       <c r="AF15" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG15" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH15" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AI15" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ15" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AK15" s="24" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="AL15" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM15" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN15" s="1">
         <f t="array" aca="1" ref="AN15" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>65476508789</v>
+        <v>53518038367</v>
       </c>
       <c r="AO15" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP15" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="AQ15" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR15" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>46191</v>
+        <v>46233</v>
       </c>
       <c r="AS15" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT15" s="28">
         <v>35591</v>
       </c>
       <c r="AU15" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV15" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW15" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX15" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY15" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ15" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA15" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB15" s="24" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="BC15" s="24" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="BD15" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE15" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF15" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG15" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH15" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI15" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ15" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK15" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL15" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM15" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN15" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO15" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP15" s="32" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="BQ15" s="33">
         <v>100</v>
       </c>
+      <c r="BR15" s="27" t="s">
+        <v>131</v>
+      </c>
     </row>
-    <row r="16" spans="1:69" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:70" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B16" s="11">
-        <v>10698471</v>
+        <v>216</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>217</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
       </c>
       <c r="J16" s="18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K16" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L16" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N16" s="18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O16" s="18">
         <v>38</v>
@@ -4596,44 +4671,44 @@
         <v>1000</v>
       </c>
       <c r="Q16" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="R16" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="S16" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="R16" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="S16" s="18" t="s">
-        <v>74</v>
-      </c>
       <c r="T16" s="20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="U16" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V16" s="18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="W16" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45795</v>
+        <v>45837</v>
       </c>
       <c r="X16" s="18" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y16" s="23" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="Z16" s="34" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="AB16" s="37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AC16" s="24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD16" s="24" t="s">
         <v>52</v>
@@ -4642,120 +4717,123 @@
         <v>35</v>
       </c>
       <c r="AF16" s="14" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AG16" s="24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AH16" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AI16" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AJ16" s="18" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AK16" s="24">
         <v>251</v>
       </c>
       <c r="AL16" s="27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AM16" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AN16" s="1">
         <f t="array" aca="1" ref="AN16" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>74989467857</v>
+        <v>74000645657</v>
       </c>
       <c r="AO16" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AP16" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AQ16" s="18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AR16" s="19" t="str">
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
       <c r="AS16" s="24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AT16" s="28">
         <v>35591</v>
       </c>
       <c r="AU16" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AV16" s="27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW16" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AX16" s="29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AY16" s="30" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AZ16" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="BA16" s="29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="BB16" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BC16" s="24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="BD16" s="14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BE16" s="27" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BF16" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BG16" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BH16" s="27" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BI16" s="27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BJ16" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BK16" s="29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BL16" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BM16" s="29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BN16" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BO16" s="29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BP16" s="32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BQ16" s="33">
         <v>100</v>
+      </c>
+      <c r="BR16" s="27" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>